<commit_message>
feat: refactor and synchronize Dual-Tone Modern Gamified SaaS UI for 12 screens and clean up mini games
</commit_message>
<xml_diff>
--- a/khao sat game/Bieu_do_Gantt_Long_Nghia.xlsx
+++ b/khao sat game/Bieu_do_Gantt_Long_Nghia.xlsx
@@ -568,7 +568,6 @@
           <t>TÊN CÔNG TY</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr"/>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -889,7 +888,7 @@
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H5" s="8" t="n"/>
@@ -956,7 +955,7 @@
       </c>
       <c r="G6" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H6" s="11" t="n"/>
@@ -1023,7 +1022,7 @@
       </c>
       <c r="G7" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H7" s="11" t="n"/>
@@ -1090,7 +1089,7 @@
       </c>
       <c r="G8" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H8" s="9" t="n"/>
@@ -1157,7 +1156,7 @@
       </c>
       <c r="G9" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H9" s="9" t="n"/>
@@ -1224,7 +1223,7 @@
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H10" s="9" t="n"/>
@@ -1291,7 +1290,7 @@
       </c>
       <c r="G11" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H11" s="9" t="n"/>
@@ -1358,7 +1357,7 @@
       </c>
       <c r="G12" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H12" s="9" t="n"/>
@@ -1425,7 +1424,7 @@
       </c>
       <c r="G13" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H13" s="9" t="n"/>
@@ -1492,7 +1491,7 @@
       </c>
       <c r="G14" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>93%</t>
         </is>
       </c>
       <c r="H14" s="9" t="n"/>
@@ -1559,7 +1558,7 @@
       </c>
       <c r="G15" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="H15" s="9" t="n"/>
@@ -1626,7 +1625,7 @@
       </c>
       <c r="G16" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="H16" s="9" t="n"/>
@@ -1693,7 +1692,7 @@
       </c>
       <c r="G17" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H17" s="9" t="n"/>
@@ -1760,7 +1759,7 @@
       </c>
       <c r="G18" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H18" s="9" t="n"/>
@@ -1827,7 +1826,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>97%</t>
         </is>
       </c>
       <c r="H19" s="9" t="n"/>
@@ -1894,7 +1893,7 @@
       </c>
       <c r="G20" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H20" s="9" t="n"/>
@@ -1961,7 +1960,7 @@
       </c>
       <c r="G21" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>90%</t>
         </is>
       </c>
       <c r="H21" s="9" t="n"/>
@@ -2028,7 +2027,7 @@
       </c>
       <c r="G22" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H22" s="9" t="n"/>
@@ -2095,7 +2094,7 @@
       </c>
       <c r="G23" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>98%</t>
         </is>
       </c>
       <c r="H23" s="9" t="n"/>
@@ -2162,7 +2161,7 @@
       </c>
       <c r="G24" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H24" s="9" t="n"/>
@@ -2229,7 +2228,7 @@
       </c>
       <c r="G25" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>95%</t>
         </is>
       </c>
       <c r="H25" s="9" t="n"/>
@@ -2296,7 +2295,7 @@
       </c>
       <c r="G26" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>100%</t>
         </is>
       </c>
       <c r="H26" s="9" t="n"/>
@@ -2363,7 +2362,7 @@
       </c>
       <c r="G27" s="6" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>77%</t>
         </is>
       </c>
       <c r="H27" s="9" t="n"/>
@@ -2430,7 +2429,7 @@
       </c>
       <c r="G28" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>85%</t>
         </is>
       </c>
       <c r="H28" s="9" t="n"/>
@@ -2497,7 +2496,7 @@
       </c>
       <c r="G29" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>75%</t>
         </is>
       </c>
       <c r="H29" s="9" t="n"/>
@@ -2564,7 +2563,7 @@
       </c>
       <c r="G30" s="10" t="inlineStr">
         <is>
-          <t>0%</t>
+          <t>70%</t>
         </is>
       </c>
       <c r="H30" s="9" t="n"/>

</xml_diff>